<commit_message>
Rescale v4 quotation line items to a 65,000 USD total
Reduce every line item proportionally so the sub total is 59,091 USD,
round the 10% production service fee to whole dollars, and land the
total excluding VAT at exactly 65,000 USD.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SvAArX2NzWcDP815G6mBWB
</commit_message>
<xml_diff>
--- a/docs/quotations/Quotation_PlanA_PLUSMIND_260915_v4.xlsx
+++ b/docs/quotations/Quotation_PlanA_PLUSMIND_260915_v4.xlsx
@@ -1356,8 +1356,8 @@
       </c>
       <c r="D18" s="27"/>
       <c r="E18" s="30" t="n">
-        <f aca="false">3*300</f>
-        <v>900</v>
+        <f aca="false">3*200</f>
+        <v>600</v>
       </c>
       <c r="F18" s="31"/>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="D19" s="27"/>
       <c r="E19" s="30" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="F19" s="31"/>
     </row>
@@ -1378,7 +1378,7 @@
       <c r="D20" s="14"/>
       <c r="E20" s="33" t="n">
         <f aca="false">SUM(E16:E19)</f>
-        <v>1400</v>
+        <v>900</v>
       </c>
       <c r="F20" s="34"/>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="D22" s="27"/>
       <c r="E22" s="30" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="F22" s="31"/>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="D23" s="27"/>
       <c r="E23" s="30" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="F23" s="31"/>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="D24" s="27"/>
       <c r="E24" s="30" t="n">
-        <v>1500</v>
+        <v>800</v>
       </c>
       <c r="F24" s="31"/>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D25" s="27"/>
       <c r="E25" s="30" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="F25" s="31"/>
     </row>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D26" s="27"/>
       <c r="E26" s="30" t="n">
-        <v>3800</v>
+        <v>2000</v>
       </c>
       <c r="F26" s="31"/>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="D27" s="27"/>
       <c r="E27" s="30" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="F27" s="31"/>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="D28" s="27"/>
       <c r="E28" s="30" t="n">
-        <v>1200</v>
+        <v>700</v>
       </c>
       <c r="F28" s="31"/>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="D29" s="27"/>
       <c r="E29" s="30" t="n">
-        <v>1300</v>
+        <v>700</v>
       </c>
       <c r="F29" s="31"/>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D30" s="27"/>
       <c r="E30" s="30" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="F30" s="31"/>
     </row>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="D31" s="27"/>
       <c r="E31" s="30" t="n">
-        <v>4200</v>
+        <v>2500</v>
       </c>
       <c r="F31" s="31"/>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="D32" s="27"/>
       <c r="E32" s="30" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="F32" s="31"/>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="D33" s="27"/>
       <c r="E33" s="30" t="n">
-        <v>700</v>
+        <v>450</v>
       </c>
       <c r="F33" s="31"/>
     </row>
@@ -1529,7 +1529,7 @@
       <c r="D34" s="14"/>
       <c r="E34" s="33" t="n">
         <f aca="false">SUM(E21:E33)</f>
-        <v>19800</v>
+        <v>11450</v>
       </c>
       <c r="F34" s="34"/>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D36" s="27"/>
       <c r="E36" s="30" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F36" s="31"/>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="D37" s="27"/>
       <c r="E37" s="30" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F37" s="31"/>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="D38" s="27"/>
       <c r="E38" s="30" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F38" s="31"/>
     </row>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="D39" s="27"/>
       <c r="E39" s="30" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F39" s="31"/>
     </row>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="D40" s="27"/>
       <c r="E40" s="30" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="F40" s="31"/>
     </row>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="D41" s="27"/>
       <c r="E41" s="30" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="F41" s="31"/>
     </row>
@@ -1614,7 +1614,7 @@
       <c r="D42" s="14"/>
       <c r="E42" s="33" t="n">
         <f aca="false">SUM(E35:E41)</f>
-        <v>10600</v>
+        <v>6200</v>
       </c>
       <c r="F42" s="34"/>
     </row>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="D44" s="27"/>
       <c r="E44" s="30" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="F44" s="31"/>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="D45" s="27"/>
       <c r="E45" s="30" t="n">
-        <v>15000</v>
+        <v>8000</v>
       </c>
       <c r="F45" s="31"/>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="D46" s="27"/>
       <c r="E46" s="30" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F46" s="31"/>
     </row>
@@ -1667,8 +1667,8 @@
       </c>
       <c r="D47" s="27"/>
       <c r="E47" s="30" t="n">
-        <f aca="false">18*200</f>
-        <v>3600</v>
+        <f aca="false">18*100</f>
+        <v>1800</v>
       </c>
       <c r="F47" s="31"/>
     </row>
@@ -1678,7 +1678,7 @@
       <c r="D48" s="14"/>
       <c r="E48" s="33" t="n">
         <f aca="false">SUM(E43:E47)</f>
-        <v>25100</v>
+        <v>13800</v>
       </c>
       <c r="F48" s="34"/>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="D50" s="27"/>
       <c r="E50" s="30" t="n">
-        <v>4500</v>
+        <v>2500</v>
       </c>
       <c r="F50" s="31"/>
     </row>
@@ -1709,8 +1709,8 @@
       </c>
       <c r="D51" s="27"/>
       <c r="E51" s="30" t="n">
-        <f aca="false">9*1500</f>
-        <v>13500</v>
+        <f aca="false">9*800</f>
+        <v>7200</v>
       </c>
       <c r="F51" s="31"/>
     </row>
@@ -1721,8 +1721,8 @@
       </c>
       <c r="D52" s="27"/>
       <c r="E52" s="30" t="n">
-        <f aca="false">8*1000</f>
-        <v>8000</v>
+        <f aca="false">8*550</f>
+        <v>4400</v>
       </c>
       <c r="F52" s="31"/>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="D53" s="27"/>
       <c r="E53" s="30" t="n">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="F53" s="31"/>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="D54" s="27"/>
       <c r="E54" s="30" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F54" s="31"/>
     </row>
@@ -1754,7 +1754,7 @@
       <c r="D55" s="14"/>
       <c r="E55" s="33" t="n">
         <f aca="false">SUM(E49:E54)</f>
-        <v>30000</v>
+        <v>16100</v>
       </c>
       <c r="F55" s="34"/>
     </row>
@@ -1774,8 +1774,8 @@
       </c>
       <c r="D57" s="27"/>
       <c r="E57" s="30" t="n">
-        <f aca="false">3*400+1500</f>
-        <v>2700</v>
+        <f aca="false">3*250+900</f>
+        <v>1650</v>
       </c>
       <c r="F57" s="31"/>
     </row>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="D58" s="27"/>
       <c r="E58" s="30" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="F58" s="31"/>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="D59" s="27"/>
       <c r="E59" s="30" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F59" s="31"/>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="D60" s="27"/>
       <c r="E60" s="30" t="n">
-        <v>1000</v>
+        <v>591</v>
       </c>
       <c r="F60" s="31"/>
     </row>
@@ -1818,7 +1818,7 @@
       <c r="D61" s="14"/>
       <c r="E61" s="33" t="n">
         <f aca="false">SUM(E56:E60)</f>
-        <v>6700</v>
+        <v>3941</v>
       </c>
       <c r="F61" s="34"/>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="D72" s="27"/>
       <c r="E72" s="30" t="n">
-        <v>3000</v>
+        <v>1800</v>
       </c>
       <c r="F72" s="31"/>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="D73" s="27"/>
       <c r="E73" s="30" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="F73" s="31"/>
     </row>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="D74" s="27"/>
       <c r="E74" s="30" t="n">
-        <v>4000</v>
+        <v>2200</v>
       </c>
       <c r="F74" s="31"/>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="D75" s="27"/>
       <c r="E75" s="30" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="F75" s="31"/>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="D77" s="27"/>
       <c r="E77" s="30" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="F77" s="31"/>
     </row>
@@ -1995,7 +1995,7 @@
       <c r="D78" s="14"/>
       <c r="E78" s="33" t="n">
         <f aca="false">SUM(E71:E77)</f>
-        <v>11400</v>
+        <v>6700</v>
       </c>
       <c r="F78" s="34"/>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="E79" s="39" t="n">
         <f aca="false">E20+E34+E42+E48+E55+E61+E69+E78</f>
-        <v>105000</v>
+        <v>59091</v>
       </c>
       <c r="F79" s="40"/>
     </row>
@@ -2018,8 +2018,8 @@
         <v>82</v>
       </c>
       <c r="E80" s="43" t="n">
-        <f aca="false">E79*0.1</f>
-        <v>10500</v>
+        <f aca="false">ROUND(E79*0.1,0)</f>
+        <v>5909</v>
       </c>
       <c r="F80" s="44"/>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="E81" s="46" t="n">
         <f aca="false">SUM(E79:E80)</f>
-        <v>115500</v>
+        <v>65000</v>
       </c>
       <c r="F81" s="47"/>
     </row>

</xml_diff>